<commit_message>
Finish translation of forecasts
</commit_message>
<xml_diff>
--- a/public/translation.xlsx
+++ b/public/translation.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2293b72959587e28/PAYT_ANALYSIS/model/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="228" documentId="8_{6AF8692F-890D-1B44-9F64-197BE6160813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{0E71E475-E12D-8E4F-BAC4-DC8AE45E9391}"/>
+  <xr:revisionPtr revIDLastSave="300" documentId="8_{6AF8692F-890D-1B44-9F64-197BE6160813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0CD88BF-FB12-A441-A664-6BB3FA9333E7}"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="12540" windowWidth="31520" windowHeight="14460" xr2:uid="{8B6CA0FD-2112-BC45-8C8C-A886CDF59FA5}"/>
+    <workbookView xWindow="240" yWindow="600" windowWidth="31520" windowHeight="26400" xr2:uid="{8B6CA0FD-2112-BC45-8C8C-A886CDF59FA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="224">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="287">
   <si>
     <t>key</t>
   </si>
@@ -783,6 +783,195 @@
 2. **Standard response**: This is the default scenario that mostly follows an extrapolation of what was observed after the last change to the fee structure. It assumes a fairly muted behavioral response to an increase in fees. However, the capacity of households to bear higher fees is assumed to fall with greater increases (even when you stagger them in multiple steps).
 3. **Strong response**: This is a scenario where we assume that compared to 2023, the financial situation of households has worsened (following inflation and increases in other national taxes). Therefore the reaction to a higher waste fee will be more pronounced this time.
 In the results, we also show a scenario of **No Policy Change**. That is, a scenario without changes to fees or other reforms that would affect revenues.</t>
+  </si>
+  <si>
+    <t>t1</t>
+  </si>
+  <si>
+    <t>Nárast poplatku v %</t>
+  </si>
+  <si>
+    <t>Fee increase in %</t>
+  </si>
+  <si>
+    <t>Odstup v rokoch</t>
+  </si>
+  <si>
+    <t>Gap in years</t>
+  </si>
+  <si>
+    <t>t2</t>
+  </si>
+  <si>
+    <t>t3</t>
+  </si>
+  <si>
+    <t>Maximálne 14d interval</t>
+  </si>
+  <si>
+    <t>Disable weekly pickup</t>
+  </si>
+  <si>
+    <t>Počet ľudí na nádobu</t>
+  </si>
+  <si>
+    <t>People per bin</t>
+  </si>
+  <si>
+    <t>t4</t>
+  </si>
+  <si>
+    <t>cr1</t>
+  </si>
+  <si>
+    <t>Coop fees</t>
+  </si>
+  <si>
+    <t>Výnosy (BD)</t>
+  </si>
+  <si>
+    <t>cr2</t>
+  </si>
+  <si>
+    <t>Coop bin count</t>
+  </si>
+  <si>
+    <t>Počet nádob (BD)</t>
+  </si>
+  <si>
+    <t>gr1</t>
+  </si>
+  <si>
+    <t>Rok</t>
+  </si>
+  <si>
+    <t>Year</t>
+  </si>
+  <si>
+    <t>gr2</t>
+  </si>
+  <si>
+    <t>Scenár</t>
+  </si>
+  <si>
+    <t>Scenario</t>
+  </si>
+  <si>
+    <t>Model</t>
+  </si>
+  <si>
+    <t>sc0</t>
+  </si>
+  <si>
+    <t>cr3</t>
+  </si>
+  <si>
+    <t>Vývoj výnosov od bytových domov a PO v EUR</t>
+  </si>
+  <si>
+    <t>Revenue from coops and businesses in EUR</t>
+  </si>
+  <si>
+    <t>cr4</t>
+  </si>
+  <si>
+    <t>Number of bins with coops and businesses</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vývoj počtu nádob v bytových domoch a PO </t>
+  </si>
+  <si>
+    <t>gr3</t>
+  </si>
+  <si>
+    <t>Platiteľ</t>
+  </si>
+  <si>
+    <t>Payee</t>
+  </si>
+  <si>
+    <t>gr4</t>
+  </si>
+  <si>
+    <t>0: Pred zmenou</t>
+  </si>
+  <si>
+    <t>0: Before change</t>
+  </si>
+  <si>
+    <t>gr5</t>
+  </si>
+  <si>
+    <t>1: Prvý rok po zmene</t>
+  </si>
+  <si>
+    <t>1: First year after change</t>
+  </si>
+  <si>
+    <t>gr6</t>
+  </si>
+  <si>
+    <t>IBV</t>
+  </si>
+  <si>
+    <t>Individual households</t>
+  </si>
+  <si>
+    <t>gr7</t>
+  </si>
+  <si>
+    <t>BD a PO</t>
+  </si>
+  <si>
+    <t>Coops and businesses</t>
+  </si>
+  <si>
+    <t>2: Posledné prognóznované obdobie</t>
+  </si>
+  <si>
+    <t>gr8</t>
+  </si>
+  <si>
+    <t>2: Last forecast period</t>
+  </si>
+  <si>
+    <t>gr9</t>
+  </si>
+  <si>
+    <t>Spolu</t>
+  </si>
+  <si>
+    <t>Together</t>
+  </si>
+  <si>
+    <t>gr10</t>
+  </si>
+  <si>
+    <t>Výnos z poplatku</t>
+  </si>
+  <si>
+    <t>Fee forecast</t>
+  </si>
+  <si>
+    <t>ir1</t>
+  </si>
+  <si>
+    <t>Vývoj výnosov z IBV v EUR</t>
+  </si>
+  <si>
+    <t>Revenue from individual homes in EUR</t>
+  </si>
+  <si>
+    <t>ir2</t>
+  </si>
+  <si>
+    <t>gr11</t>
+  </si>
+  <si>
+    <t>Počet nádob</t>
+  </si>
+  <si>
+    <t>Bin count</t>
   </si>
 </sst>
 </file>
@@ -1170,7 +1359,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F81EA9-A9C7-6E4A-8243-CC330D585D50}">
-  <dimension ref="A1:C86"/>
+  <dimension ref="A1:C109"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="93.83203125" customWidth="1"/>
@@ -1980,6 +2169,17 @@
         <v>209</v>
       </c>
     </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A83" t="s">
+        <v>249</v>
+      </c>
+      <c r="B83" t="s">
+        <v>246</v>
+      </c>
+      <c r="C83" t="s">
+        <v>247</v>
+      </c>
+    </row>
     <row r="84" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>210</v>
@@ -2011,6 +2211,231 @@
       </c>
       <c r="C86" t="s">
         <v>218</v>
+      </c>
+    </row>
+    <row r="88" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A88" t="s">
+        <v>224</v>
+      </c>
+      <c r="B88" t="s">
+        <v>225</v>
+      </c>
+      <c r="C88" t="s">
+        <v>226</v>
+      </c>
+    </row>
+    <row r="89" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A89" t="s">
+        <v>229</v>
+      </c>
+      <c r="B89" t="s">
+        <v>227</v>
+      </c>
+      <c r="C89" t="s">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="90" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A90" t="s">
+        <v>230</v>
+      </c>
+      <c r="B90" t="s">
+        <v>231</v>
+      </c>
+      <c r="C90" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A91" t="s">
+        <v>235</v>
+      </c>
+      <c r="B91" t="s">
+        <v>233</v>
+      </c>
+      <c r="C91" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="93" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A93" t="s">
+        <v>236</v>
+      </c>
+      <c r="B93" t="s">
+        <v>238</v>
+      </c>
+      <c r="C93" t="s">
+        <v>237</v>
+      </c>
+    </row>
+    <row r="94" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A94" t="s">
+        <v>239</v>
+      </c>
+      <c r="B94" t="s">
+        <v>241</v>
+      </c>
+      <c r="C94" t="s">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A95" t="s">
+        <v>250</v>
+      </c>
+      <c r="B95" t="s">
+        <v>251</v>
+      </c>
+      <c r="C95" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="96" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A96" t="s">
+        <v>253</v>
+      </c>
+      <c r="B96" t="s">
+        <v>255</v>
+      </c>
+      <c r="C96" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="97" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A97" t="s">
+        <v>242</v>
+      </c>
+      <c r="B97" t="s">
+        <v>243</v>
+      </c>
+      <c r="C97" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="98" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A98" t="s">
+        <v>245</v>
+      </c>
+      <c r="B98" t="s">
+        <v>248</v>
+      </c>
+      <c r="C98" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="99" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A99" t="s">
+        <v>256</v>
+      </c>
+      <c r="B99" t="s">
+        <v>257</v>
+      </c>
+      <c r="C99" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="100" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A100" t="s">
+        <v>259</v>
+      </c>
+      <c r="B100" t="s">
+        <v>260</v>
+      </c>
+      <c r="C100" t="s">
+        <v>261</v>
+      </c>
+    </row>
+    <row r="101" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A101" t="s">
+        <v>262</v>
+      </c>
+      <c r="B101" t="s">
+        <v>263</v>
+      </c>
+      <c r="C101" t="s">
+        <v>264</v>
+      </c>
+    </row>
+    <row r="102" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A102" t="s">
+        <v>265</v>
+      </c>
+      <c r="B102" t="s">
+        <v>266</v>
+      </c>
+      <c r="C102" t="s">
+        <v>267</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A103" t="s">
+        <v>268</v>
+      </c>
+      <c r="B103" t="s">
+        <v>269</v>
+      </c>
+      <c r="C103" t="s">
+        <v>270</v>
+      </c>
+    </row>
+    <row r="104" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A104" t="s">
+        <v>272</v>
+      </c>
+      <c r="B104" t="s">
+        <v>271</v>
+      </c>
+      <c r="C104" t="s">
+        <v>273</v>
+      </c>
+    </row>
+    <row r="105" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A105" t="s">
+        <v>274</v>
+      </c>
+      <c r="B105" t="s">
+        <v>275</v>
+      </c>
+      <c r="C105" t="s">
+        <v>276</v>
+      </c>
+    </row>
+    <row r="106" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A106" t="s">
+        <v>277</v>
+      </c>
+      <c r="B106" t="s">
+        <v>278</v>
+      </c>
+      <c r="C106" t="s">
+        <v>279</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A107" t="s">
+        <v>284</v>
+      </c>
+      <c r="B107" t="s">
+        <v>285</v>
+      </c>
+      <c r="C107" t="s">
+        <v>286</v>
+      </c>
+    </row>
+    <row r="108" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A108" t="s">
+        <v>280</v>
+      </c>
+      <c r="B108" t="s">
+        <v>281</v>
+      </c>
+      <c r="C108" t="s">
+        <v>282</v>
+      </c>
+    </row>
+    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A109" t="s">
+        <v>283</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Finish translation of expenses
</commit_message>
<xml_diff>
--- a/public/translation.xlsx
+++ b/public/translation.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/2293b72959587e28/PAYT_ANALYSIS/model/public/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="300" documentId="8_{6AF8692F-890D-1B44-9F64-197BE6160813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{C0CD88BF-FB12-A441-A664-6BB3FA9333E7}"/>
+  <xr:revisionPtr revIDLastSave="317" documentId="8_{6AF8692F-890D-1B44-9F64-197BE6160813}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27BD6503-F2E8-C244-AD0A-18F8313AFDF6}"/>
   <bookViews>
     <workbookView xWindow="240" yWindow="600" windowWidth="31520" windowHeight="26400" xr2:uid="{8B6CA0FD-2112-BC45-8C8C-A886CDF59FA5}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="292" uniqueCount="287">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="306" uniqueCount="301">
   <si>
     <t>key</t>
   </si>
@@ -962,9 +962,6 @@
     <t>Revenue from individual homes in EUR</t>
   </si>
   <si>
-    <t>ir2</t>
-  </si>
-  <si>
     <t>gr11</t>
   </si>
   <si>
@@ -972,6 +969,51 @@
   </si>
   <si>
     <t>Bin count</t>
+  </si>
+  <si>
+    <t>olo1</t>
+  </si>
+  <si>
+    <t>2 Ostatné náklady</t>
+  </si>
+  <si>
+    <t>2 Other expenses</t>
+  </si>
+  <si>
+    <t>olo2</t>
+  </si>
+  <si>
+    <t>4 OLO Zberné dvory</t>
+  </si>
+  <si>
+    <t>4 OLO Waste yards</t>
+  </si>
+  <si>
+    <t>olo3</t>
+  </si>
+  <si>
+    <t>3 Podiel MČ</t>
+  </si>
+  <si>
+    <t>3 City district share</t>
+  </si>
+  <si>
+    <t>olo4</t>
+  </si>
+  <si>
+    <t>Kategória</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>olo5</t>
+  </si>
+  <si>
+    <t>Náklady</t>
+  </si>
+  <si>
+    <t>Expenses</t>
   </si>
 </sst>
 </file>
@@ -1359,7 +1401,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D5F81EA9-A9C7-6E4A-8243-CC330D585D50}">
-  <dimension ref="A1:C109"/>
+  <dimension ref="A1:C114"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="2" max="2" width="93.83203125" customWidth="1"/>
@@ -2413,13 +2455,13 @@
     </row>
     <row r="107" spans="1:3" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
+        <v>283</v>
+      </c>
+      <c r="B107" t="s">
         <v>284</v>
       </c>
-      <c r="B107" t="s">
+      <c r="C107" t="s">
         <v>285</v>
-      </c>
-      <c r="C107" t="s">
-        <v>286</v>
       </c>
     </row>
     <row r="108" spans="1:3" x14ac:dyDescent="0.2">
@@ -2433,9 +2475,59 @@
         <v>282</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.2">
-      <c r="A109" t="s">
-        <v>283</v>
+    <row r="110" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A110" t="s">
+        <v>286</v>
+      </c>
+      <c r="B110" t="s">
+        <v>287</v>
+      </c>
+      <c r="C110" t="s">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="111" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A111" t="s">
+        <v>289</v>
+      </c>
+      <c r="B111" t="s">
+        <v>290</v>
+      </c>
+      <c r="C111" t="s">
+        <v>291</v>
+      </c>
+    </row>
+    <row r="112" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A112" t="s">
+        <v>292</v>
+      </c>
+      <c r="B112" t="s">
+        <v>293</v>
+      </c>
+      <c r="C112" t="s">
+        <v>294</v>
+      </c>
+    </row>
+    <row r="113" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A113" t="s">
+        <v>295</v>
+      </c>
+      <c r="B113" t="s">
+        <v>296</v>
+      </c>
+      <c r="C113" t="s">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="114" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A114" t="s">
+        <v>298</v>
+      </c>
+      <c r="B114" t="s">
+        <v>299</v>
+      </c>
+      <c r="C114" t="s">
+        <v>300</v>
       </c>
     </row>
   </sheetData>

</xml_diff>